<commit_message>
the InvestmentBlock form writes a modular extendable asset with an integer design too, the number of its modules, and solves it with the BundleSolver of InvestmentBlock/BSPar-int.txt
</commit_message>
<xml_diff>
--- a/pypsa2smspp/data/smspp_parameters.xlsx
+++ b/pypsa2smspp/data/smspp_parameters.xlsx
@@ -3094,7 +3094,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="17" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -3266,46 +3266,44 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>InvestmentCost</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Capital cost if only lines</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="inlineStr">
-        <is>
-          <t>Parameter</t>
-        </is>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>[NDL] | [NDLL] | [NDLLi]</t>
-        </is>
-      </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1 if the design counts modules</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>[Nass]</t>
+        </is>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>MinCapacityDesign</t>
+          <t>InvestmentCost</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Minimum acceptable size</t>
+          <t>Capital cost if only lines</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
@@ -3332,30 +3330,62 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>MinCapacityDesign</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Minimum acceptable size</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>[NDL] | [NDLL] | [NDLLi]</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>MaxCapacityDesign</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Maximum acceptable size</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
-        <is>
-          <t>Parameter</t>
-        </is>
-      </c>
-      <c r="D8" s="1" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E8" s="1" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>[NDL] | [NDLL] | [NDLLi]</t>
         </is>
       </c>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="F9" s="1" t="inlineStr">
         <is>
           <t>False</t>
         </is>

</xml_diff>

<commit_message>
a Store is written with no power limit and no converter, its power being bounded by its levels and by the Links around it, and the turbine of a StorageUnit with ExactFlowToPower, so that the model of SMS++ is the one of PyPSA
</commit_message>
<xml_diff>
--- a/pypsa2smspp/data/smspp_parameters.xlsx
+++ b/pypsa2smspp/data/smspp_parameters.xlsx
@@ -2308,7 +2308,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16.6640625" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -2828,46 +2828,46 @@
       </c>
     </row>
     <row r="17" ht="18.75" customHeight="1" s="6">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>LinearTerm</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
-        <is>
-          <t>Linear multiplier of FTAP function</t>
-        </is>
-      </c>
-      <c r="C17" s="1" t="inlineStr">
-        <is>
-          <t>Parameter</t>
-        </is>
-      </c>
-      <c r="D17" s="1" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>[NP] | [T][NP]</t>
-        </is>
-      </c>
-      <c r="F17" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ExactFlowToPower</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Single-piece turbine producing exactly the power of its piece</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>[NA]</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>True</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18.75" customHeight="1" s="6">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>DeltaRampUp</t>
+          <t>LinearTerm</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>Ramp-up limit</t>
+          <t>Linear multiplier of FTAP function</t>
         </is>
       </c>
       <c r="C18" s="1" t="inlineStr">
@@ -2882,24 +2882,24 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>[NA] | [T][NA]</t>
+          <t>[NP] | [T][NP]</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18.75" customHeight="1" s="6">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>DeltaRampDown</t>
+          <t>DeltaRampUp</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>Ramp-down limit</t>
+          <t>Ramp-up limit</t>
         </is>
       </c>
       <c r="C19" s="1" t="inlineStr">
@@ -2926,12 +2926,12 @@
     <row r="20" ht="18.75" customHeight="1" s="6">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>DownhillFlow</t>
+          <t>DeltaRampDown</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>Downhill flow rate</t>
+          <t>Ramp-down limit</t>
         </is>
       </c>
       <c r="C20" s="1" t="inlineStr">
@@ -2941,12 +2941,12 @@
       </c>
       <c r="D20" s="1" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>float</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>[NA]</t>
+          <t>[NA] | [T][NA]</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
@@ -2958,12 +2958,12 @@
     <row r="21" ht="18.75" customHeight="1" s="6">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>UphillFlow</t>
+          <t>DownhillFlow</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>Uphill flow rate</t>
+          <t>Downhill flow rate</t>
         </is>
       </c>
       <c r="C21" s="1" t="inlineStr">
@@ -2990,12 +2990,12 @@
     <row r="22" ht="18.75" customHeight="1" s="6">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>InertiaPower</t>
+          <t>UphillFlow</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t>Inertia power</t>
+          <t>Uphill flow rate</t>
         </is>
       </c>
       <c r="C22" s="1" t="inlineStr">
@@ -3005,12 +3005,12 @@
       </c>
       <c r="D22" s="1" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>[NA] | [T][NA]</t>
+          <t>[NA]</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
@@ -3022,12 +3022,12 @@
     <row r="23" ht="18.75" customHeight="1" s="6">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>InitialFlowRate</t>
+          <t>InertiaPower</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t>Initial flow rate</t>
+          <t>Inertia power</t>
         </is>
       </c>
       <c r="C23" s="1" t="inlineStr">
@@ -3042,7 +3042,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>[NA]</t>
+          <t>[NA] | [T][NA]</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
@@ -3054,30 +3054,62 @@
     <row r="24" ht="18.75" customHeight="1" s="6">
       <c r="A24" s="1" t="inlineStr">
         <is>
+          <t>InitialFlowRate</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>Initial flow rate</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>[NA]</t>
+        </is>
+      </c>
+      <c r="F24" s="1" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
           <t>InitialVolumetric</t>
         </is>
       </c>
-      <c r="B24" s="1" t="inlineStr">
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>Initial volumetric</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
-        <is>
-          <t>Parameter</t>
-        </is>
-      </c>
-      <c r="D24" s="1" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="C25" s="1" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="D25" s="1" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>[NR]</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="F25" s="1" t="inlineStr">
         <is>
           <t>False</t>
         </is>

</xml_diff>

<commit_message>
MaxVolumetric and MinVolumetric of a hydro unit written as [NumberReservoirs][TimeHorizon], the order HydroUnitBlock reads; they were transposed, which SMS++ corrected only with a single reservoir
</commit_message>
<xml_diff>
--- a/pypsa2smspp/data/smspp_parameters.xlsx
+++ b/pypsa2smspp/data/smspp_parameters.xlsx
@@ -2498,7 +2498,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>[1][NR] | [T][NR]</t>
+          <t>[1][NR] | [NR][T]</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
@@ -2530,7 +2530,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>[1][NR] | [T][NR]</t>
+          <t>[1][NR] | [NR][T]</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Revert "Changes for the BundleSolver 2.0 (#62)"
This reverts commit c881cf781fd150f50ab71c0a259736d94cca336e.
</commit_message>
<xml_diff>
--- a/pypsa2smspp/data/smspp_parameters.xlsx
+++ b/pypsa2smspp/data/smspp_parameters.xlsx
@@ -3094,7 +3094,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="17" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -3266,44 +3266,46 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Integer</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>1 if the design counts modules</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Parameter</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>[Nass]</t>
-        </is>
-      </c>
-      <c r="F6" t="b">
-        <v>1</v>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>InvestmentCost</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Capital cost if only lines</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>[NDL] | [NDLL] | [NDLLi]</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>InvestmentCost</t>
+          <t>MinCapacityDesign</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Capital cost if only lines</t>
+          <t>Minimum acceptable size</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
@@ -3330,12 +3332,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>MinCapacityDesign</t>
+          <t>MaxCapacityDesign</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Minimum acceptable size</t>
+          <t>Maximum acceptable size</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
@@ -3354,38 +3356,6 @@
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>MaxCapacityDesign</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Maximum acceptable size</t>
-        </is>
-      </c>
-      <c r="C9" s="1" t="inlineStr">
-        <is>
-          <t>Parameter</t>
-        </is>
-      </c>
-      <c r="D9" s="1" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E9" s="1" t="inlineStr">
-        <is>
-          <t>[NDL] | [NDLL] | [NDLLi]</t>
-        </is>
-      </c>
-      <c r="F9" s="1" t="inlineStr">
         <is>
           <t>False</t>
         </is>

</xml_diff>

<commit_message>
Revert "Changes for the BundleSolver 2.0 (#62)" (#74)
This reverts commit c881cf781fd150f50ab71c0a259736d94cca336e.
</commit_message>
<xml_diff>
--- a/pypsa2smspp/data/smspp_parameters.xlsx
+++ b/pypsa2smspp/data/smspp_parameters.xlsx
@@ -3094,7 +3094,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="17" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -3266,44 +3266,46 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Integer</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>1 if the design counts modules</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Parameter</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>[Nass]</t>
-        </is>
-      </c>
-      <c r="F6" t="b">
-        <v>1</v>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>InvestmentCost</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Capital cost if only lines</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>[NDL] | [NDLL] | [NDLLi]</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>InvestmentCost</t>
+          <t>MinCapacityDesign</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Capital cost if only lines</t>
+          <t>Minimum acceptable size</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
@@ -3330,12 +3332,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>MinCapacityDesign</t>
+          <t>MaxCapacityDesign</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Minimum acceptable size</t>
+          <t>Maximum acceptable size</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
@@ -3354,38 +3356,6 @@
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>MaxCapacityDesign</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Maximum acceptable size</t>
-        </is>
-      </c>
-      <c r="C9" s="1" t="inlineStr">
-        <is>
-          <t>Parameter</t>
-        </is>
-      </c>
-      <c r="D9" s="1" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E9" s="1" t="inlineStr">
-        <is>
-          <t>[NDL] | [NDLL] | [NDLLi]</t>
-        </is>
-      </c>
-      <c r="F9" s="1" t="inlineStr">
         <is>
           <t>False</t>
         </is>

</xml_diff>